<commit_message>
docs(order-management): mark 24.1-24.4 shipped (SBE-1125 GET /api/v1/orders)
Update Implementation Status (md + xlsx) for the four consolidated-list
stories now that the endpoint is built, smoke-tested, reviewed, and green:

- Branch SBE-1125; commits 6dc3104 (feat) + b95627b (SonarQube S7781 fix);
  PR #513 -> dev; pipeline #838 SUCCESSFUL; Swagger tag Admin - Order Management.
- md: rewrite Implementation Status to the filled lifecycle format with a
  per-requirement done/blocked/delegated table; refresh the Implementation line.
- xlsx: fill Overview lifecycle fields, rebuild the Implementation Status sheet,
  and fill the per-req Impl Status column (header dated 2026-07-02).

Status: 24.1 12/14 (24.1-b booth-build Blocked, 24.1-e Delegated -> 24.5);
24.2 all 8 filters (24.2-d Delegated -> GET /api/v1/cities); 24.3 all 7 search;
24.4 all 3 sorting.
</commit_message>
<xml_diff>
--- a/order_management/24.1-view-and-manage-all-orders/24.1 - View and manage all orders.xlsx
+++ b/order_management/24.1-view-and-manage-all-orders/24.1 - View and manage all orders.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +43,12 @@
       <color rgb="000563C1"/>
       <u val="single"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -96,6 +100,11 @@
         <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -137,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -195,6 +204,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -710,7 +725,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Not started — analysis only</t>
+          <t>12 of 14 reqs shipped in SBE-1125 (GET /api/v1/orders); 24.1-b Blocked (booth-build), 24.1-e Delegated → 24.5 (SBE-1129)</t>
         </is>
       </c>
     </row>
@@ -722,7 +737,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SBE-1125 (admin-backend-api)</t>
         </is>
       </c>
     </row>
@@ -734,7 +749,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6dc3104 (feat — OM list endpoint), b95627b (SonarQube S7781 fix)</t>
         </is>
       </c>
     </row>
@@ -746,7 +761,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Bitbucket #513 → dev</t>
         </is>
       </c>
     </row>
@@ -836,7 +851,7 @@
       </c>
       <c r="L1" s="9" t="inlineStr">
         <is>
-          <t>Impl Status (2026-07-01)</t>
+          <t>Impl Status (2026-07-02)</t>
         </is>
       </c>
     </row>
@@ -892,9 +907,9 @@
           <t>Open §Order Management → Story 24.1</t>
         </is>
       </c>
-      <c r="L2" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started</t>
+      <c r="L2" s="20" t="inlineStr">
+        <is>
+          <t>✅ Done — GET /api/v1/orders (paginated, product-scoped, wrapped envelope).</t>
         </is>
       </c>
     </row>
@@ -950,9 +965,9 @@
           <t>Open §Order Management → Story 24.1</t>
         </is>
       </c>
-      <c r="L3" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started (Blocked — Booth Build feature (deferred) must ship an order-creation write-path before booth-build orders can appear.)</t>
+      <c r="L3" s="20" t="inlineStr">
+        <is>
+          <t>⛔ Blocked — no booth-build producer (SBE-1304/1399/1088); list auto-surfaces once one writes order_type=product.</t>
         </is>
       </c>
     </row>
@@ -1008,9 +1023,9 @@
           <t>Open §Order Management → Story 24.1</t>
         </is>
       </c>
-      <c r="L4" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started</t>
+      <c r="L4" s="20" t="inlineStr">
+        <is>
+          <t>✅ Done — row id + order_number + customer_name (billing snapshot).</t>
         </is>
       </c>
     </row>
@@ -1066,9 +1081,9 @@
           <t>Open §Order Management → Story 24.1</t>
         </is>
       </c>
-      <c r="L5" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started</t>
+      <c r="L5" s="20" t="inlineStr">
+        <is>
+          <t>✅ Done — company_name = billing_company_name (blank → Company.name fallback).</t>
         </is>
       </c>
     </row>
@@ -1124,9 +1139,9 @@
           <t>Open §Order Management → Story 24.1</t>
         </is>
       </c>
-      <c r="L6" s="15" t="inlineStr">
-        <is>
-          <t>Delegated → 24.5 Quick Actions Per Order Item (SBE-1129, In Progress); 24.1 only returns the row id</t>
+      <c r="L6" s="20" t="inlineStr">
+        <is>
+          <t>Delegated → 24.5 Quick Actions (SBE-1129) — list returns row id only.</t>
         </is>
       </c>
     </row>
@@ -1182,9 +1197,9 @@
           <t>Open §Order Management → Story 24.1</t>
         </is>
       </c>
-      <c r="L7" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started</t>
+      <c r="L7" s="20" t="inlineStr">
+        <is>
+          <t>✅ Done — item_total = Order.total (2-dp string).</t>
         </is>
       </c>
     </row>
@@ -1240,9 +1255,9 @@
           <t>Open §Order Management → Story 24.1</t>
         </is>
       </c>
-      <c r="L8" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started</t>
+      <c r="L8" s="20" t="inlineStr">
+        <is>
+          <t>✅ Done — balance_due = total − paid_amount, floored at 0.</t>
         </is>
       </c>
     </row>
@@ -1298,9 +1313,9 @@
           <t>Open §Order Management → Story 24.1</t>
         </is>
       </c>
-      <c r="L9" s="15" t="inlineStr">
-        <is>
-          <t>Deliverable — deduped shows[] array (multi-show resolved 2026-07-02).</t>
+      <c r="L9" s="20" t="inlineStr">
+        <is>
+          <t>✅ Done — deduped shows[] (id/title/city/date), [] when none.</t>
         </is>
       </c>
     </row>
@@ -1356,9 +1371,9 @@
           <t>Open §Order Management → Story 24.1</t>
         </is>
       </c>
-      <c r="L10" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started</t>
+      <c r="L10" s="20" t="inlineStr">
+        <is>
+          <t>✅ Done — sales_person (User join), null for self-service.</t>
         </is>
       </c>
     </row>
@@ -1414,9 +1429,9 @@
           <t>Open §Order Management → Story 24.1</t>
         </is>
       </c>
-      <c r="L11" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started</t>
+      <c r="L11" s="20" t="inlineStr">
+        <is>
+          <t>✅ Done — sales_channel from cart.created_by_type (exhibitor→self_service, else admin_sales).</t>
         </is>
       </c>
     </row>
@@ -1472,9 +1487,9 @@
           <t>Open §Order Management → Story 24.1</t>
         </is>
       </c>
-      <c r="L12" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started</t>
+      <c r="L12" s="20" t="inlineStr">
+        <is>
+          <t>✅ Done — order_date = Order.created_at.</t>
         </is>
       </c>
     </row>
@@ -1530,9 +1545,9 @@
           <t>Open §Order Management → Story 24.1</t>
         </is>
       </c>
-      <c r="L13" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started</t>
+      <c r="L13" s="20" t="inlineStr">
+        <is>
+          <t>✅ Done — selectable rows surfaced via row id.</t>
         </is>
       </c>
     </row>
@@ -1588,9 +1603,9 @@
           <t>Open §Order Management → Story 24.1</t>
         </is>
       </c>
-      <c r="L14" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started</t>
+      <c r="L14" s="20" t="inlineStr">
+        <is>
+          <t>✅ Done — @Permissions('orders.list') + JWT guard; orders.list seeded (Admin + Super Administrator).</t>
         </is>
       </c>
     </row>
@@ -1646,9 +1661,9 @@
           <t>Open §Order Management → Story 24.1</t>
         </is>
       </c>
-      <c r="L15" s="15" t="inlineStr">
-        <is>
-          <t>Deliverable — authoritative figures on Order.total/paid_amount (resolved 2026-07-02).</t>
+      <c r="L15" s="20" t="inlineStr">
+        <is>
+          <t>✅ Done — authoritative Order.total/paid_amount (no standalone billing service).</t>
         </is>
       </c>
     </row>
@@ -1912,274 +1927,190 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="B1" s="16" t="inlineStr">
+      <c r="B1" s="21" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
-        <is>
-          <t>Not started — analysis/feasibility stage only; no branch or SBE ticket cut yet. Extended tracking format applied; per-requirement build status is ◻ Not started.</t>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>Shipped — built, live-smoke-tested, code-reviewed; all gates green; PR open against dev (not yet merged).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>Branch / PR</t>
-        </is>
-      </c>
-      <c r="B3" s="15" t="inlineStr">
-        <is>
-          <t>— (not started). No SBE ticket / PR / Swagger tag yet.</t>
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>SBE-1125 (admin-backend-api)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.1-a</t>
-        </is>
-      </c>
-      <c r="B4" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — OM list endpoint (GET /api/v1/orders).</t>
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>SBE ticket</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>SBE-1125</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Commits</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>6dc3104 (feat — OM list endpoint), b95627b (SonarQube S7781 fix)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Bitbucket #513 → dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Swagger tag</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Admin - Order Management (/api/docs/admin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Build gates</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Pipeline #838 SUCCESSFUL — gitleaks + lint/typecheck/test (2702 pass; orders module 48) + SonarQube quality gate all green</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Live smoke</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>RBAC/validation matrix + 32-assertion self-cleaning seeded fixture (exhibitor/admin/null-cart orders, subscription exclusion, derivations, filters, sort, search) — all passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>Confirmed build scope</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>GET /api/v1/orders — 24.1-a,c,d,f,g,h,i,j,k,l,m,n shipped (12 of 14). Row: id, order_number, customer_name, company_name, item_total, balance_due, shows[], sales_person, sales_channel, order_date, status, currency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Remaining — 24.1-b</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started (Blocked) — include booth-build orders; no producer exists (see Deferred Work).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.1-c</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — Order ID + Customer Name clickable cell.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.1-d</t>
-        </is>
-      </c>
-      <c r="B7" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — Company Name column.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.1-f</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — Item Total column.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.1-g</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — Balance Due column.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.1-h</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — Show column (multi-show behavior pending).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.1-i</t>
-        </is>
-      </c>
-      <c r="B11" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — Sales Person column.</t>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Blocked — booth-build orders; no producer (SBE-1304/1399/1088). No OM-list change needed: the list surfaces the order once it lands as order_type=product.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.1-j</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — Sales Channel column.</t>
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Delegated — 24.1-e</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Quick Links → story 24.5 Quick Actions Per Order Item (SBE-1129, In Progress); the list only returns the row id.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.1-k</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — Date column.</t>
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Dependency — Booth Build</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Booth Build order producer (write-path creating booth-build orders) — needed for 24.1-b. Owner: SBE-1304/1399/1088 (deferred).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.1-l</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — Per-row selection checkbox.</t>
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Dependency — Order Details</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>24.1-c click destination page — owner: OM Order Details story; the list owes only row id/order_number (shipped).</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.1-m</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started — Backend-enforced list data / access (RBAC).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — 24.1-n</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="inlineStr">
-        <is>
-          <t>◻ Not started (Partial) — Total/Balance Due column-accuracy source; figures authoritative but no standalone billing service.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>Open decision — Show column</t>
-        </is>
-      </c>
-      <c r="B17" s="15" t="inlineStr">
-        <is>
-          <t>Multi-show "Show" column behavior (join names / "Multiple" / single-show scoping). Gates 24.1-h.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="15" t="inlineStr">
-        <is>
-          <t>Open decision — Billing service</t>
-        </is>
-      </c>
-      <c r="B18" s="15" t="inlineStr">
-        <is>
-          <t>'Centralized billing service' literal vs authoritative. Gates 24.1-n. Figures live on Order.total/paid_amount.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>Dependency — Booth Build</t>
-        </is>
-      </c>
-      <c r="B19" s="15" t="inlineStr">
-        <is>
-          <t>A Booth Build order producer (write-path creating booth-build orders) — needed for 24.1-b. Owner: Order Management / Booth Build (deferred feature).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="15" t="inlineStr">
-        <is>
-          <t>Dependency — Quick Actions (Delegated → 24.5)</t>
-        </is>
-      </c>
-      <c r="B20" s="15" t="inlineStr">
-        <is>
-          <t>Per-row quick-action behaviour (24.1-e, Delegated to 24.5 Quick Actions, SBE-1129, In Progress). Owner: story 24.5 "Quick Actions Per Order Item"; list returns only the row id.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>Dependency — Order Details</t>
-        </is>
-      </c>
-      <c r="B21" s="15" t="inlineStr">
-        <is>
-          <t>24.1-c click destination page. Owner: separate OM Order Details story; 24.1 owes only the row id/order_number.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Out of API scope</t>
         </is>
       </c>
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>Front-end row-to-detail / action / checkbox wiring and anything Delegated or out of scope are outside API scope.</t>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>Front-end row-to-detail / action / checkbox wiring.</t>
         </is>
       </c>
     </row>

</xml_diff>